<commit_message>
docs: correct Flyer pause reason codes in HMI reference
Flyer Frame sheet had stale Pause Reason values
(3=LiftFault,4=BobbinFull). Updated to match confirmed firmware
defines (2=FrontSensorCut,4=Lapping,5=BackSensorCut; code 3 unused)
and noted the correction so the old value isn't mistaken for
current again.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Gen4_Spinning_HMI_v8.xlsx
+++ b/Gen4_Spinning_HMI_v8.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Frame Format" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Opcodes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Draw Frame" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Carding (Blow Card)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Flyer Frame" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Ring Doubler" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Diagnostics" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Carousel" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="PID" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Defaults &amp; Limits" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Quick Reference" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Format" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opcodes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Draw Frame" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carding (Blow Card)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flyer Frame" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ring Doubler" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diagnostics" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carousel" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PID" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defaults &amp; Limits" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Reference" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -142,7 +142,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -156,11 +156,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -264,6 +292,8 @@
     <xf numFmtId="0" fontId="3" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -652,6 +682,10 @@
           <t>BT Frame Structure  (all values in hex ASCII, upper-case)</t>
         </is>
       </c>
+      <c r="B2" s="35" t="n"/>
+      <c r="C2" s="35" t="n"/>
+      <c r="D2" s="35" t="n"/>
+      <c r="E2" s="36" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -875,6 +909,10 @@
           <t>Frame Length Calculation</t>
         </is>
       </c>
+      <c r="B12" s="35" t="n"/>
+      <c r="C12" s="35" t="n"/>
+      <c r="D12" s="35" t="n"/>
+      <c r="E12" s="36" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -920,6 +958,10 @@
           <t>TLV Encoding  (Type-Length-Value)</t>
         </is>
       </c>
+      <c r="B16" s="35" t="n"/>
+      <c r="C16" s="35" t="n"/>
+      <c r="D16" s="35" t="n"/>
+      <c r="E16" s="36" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1023,6 +1065,10 @@
           <t>TLV Data Types — Wire Encoding</t>
         </is>
       </c>
+      <c r="B22" s="35" t="n"/>
+      <c r="C22" s="35" t="n"/>
+      <c r="D22" s="35" t="n"/>
+      <c r="E22" s="36" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1138,6 +1184,10 @@
           <t>Special Strings (not BT frames — raw ASCII)</t>
         </is>
       </c>
+      <c r="B28" s="35" t="n"/>
+      <c r="C28" s="35" t="n"/>
+      <c r="D28" s="35" t="n"/>
+      <c r="E28" s="36" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
@@ -1280,6 +1330,10 @@
           <t>BT Connection Handshake</t>
         </is>
       </c>
+      <c r="B35" s="35" t="n"/>
+      <c r="C35" s="35" t="n"/>
+      <c r="D35" s="35" t="n"/>
+      <c r="E35" s="36" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
@@ -1447,6 +1501,10 @@
           <t>Draw Frame (DF) — Settings Defaults &amp; Limits</t>
         </is>
       </c>
+      <c r="B2" s="35" t="n"/>
+      <c r="C2" s="35" t="n"/>
+      <c r="D2" s="35" t="n"/>
+      <c r="E2" s="36" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -1643,6 +1701,10 @@
           <t>Draw Frame — AL Settings Limits (opcode 0x11 TLVs)</t>
         </is>
       </c>
+      <c r="B11" s="35" t="n"/>
+      <c r="C11" s="35" t="n"/>
+      <c r="D11" s="35" t="n"/>
+      <c r="E11" s="36" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -1812,6 +1874,10 @@
           <t>Carding (Blow Card) — Settings Defaults &amp; Limits</t>
         </is>
       </c>
+      <c r="B19" s="35" t="n"/>
+      <c r="C19" s="35" t="n"/>
+      <c r="D19" s="35" t="n"/>
+      <c r="E19" s="36" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -2062,6 +2128,10 @@
           <t>Flyer Frame — Settings Defaults &amp; Limits</t>
         </is>
       </c>
+      <c r="B30" s="35" t="n"/>
+      <c r="C30" s="35" t="n"/>
+      <c r="D30" s="35" t="n"/>
+      <c r="E30" s="36" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="24" t="inlineStr">
@@ -2447,6 +2517,10 @@
           <t>Ring Doubler — Settings Defaults &amp; Limits</t>
         </is>
       </c>
+      <c r="B46" s="35" t="n"/>
+      <c r="C46" s="35" t="n"/>
+      <c r="D46" s="35" t="n"/>
+      <c r="E46" s="36" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
@@ -5332,6 +5406,11 @@
           <t>Machine Substates (used in opcode 0x06 SS field)</t>
         </is>
       </c>
+      <c r="B25" s="35" t="n"/>
+      <c r="C25" s="35" t="n"/>
+      <c r="D25" s="35" t="n"/>
+      <c r="E25" s="35" t="n"/>
+      <c r="F25" s="36" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
@@ -5513,6 +5592,12 @@
           <t>1. Settings From App  |  opcode 0x01  |  substate 0x01  |  App → Board  |  Save to EEPROM</t>
         </is>
       </c>
+      <c r="B2" s="35" t="n"/>
+      <c r="C2" s="35" t="n"/>
+      <c r="D2" s="35" t="n"/>
+      <c r="E2" s="35" t="n"/>
+      <c r="F2" s="35" t="n"/>
+      <c r="G2" s="36" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -5779,6 +5864,12 @@
           <t>2. Settings To App  |  opcode 0x02  |  Board → App  |  Same TLVs as above, sent on GET or after save</t>
         </is>
       </c>
+      <c r="B11" s="35" t="n"/>
+      <c r="C11" s="35" t="n"/>
+      <c r="D11" s="35" t="n"/>
+      <c r="E11" s="35" t="n"/>
+      <c r="F11" s="35" t="n"/>
+      <c r="G11" s="36" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -5799,6 +5890,12 @@
           <t>3. Machine State  |  opcode 0x06  |  Board → App  |  Live status — sent periodically while running</t>
         </is>
       </c>
+      <c r="B14" s="35" t="n"/>
+      <c r="C14" s="35" t="n"/>
+      <c r="D14" s="35" t="n"/>
+      <c r="E14" s="35" t="n"/>
+      <c r="F14" s="35" t="n"/>
+      <c r="G14" s="36" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
@@ -5806,6 +5903,12 @@
           <t xml:space="preserve">   3a. Running State (SS = 0x01)</t>
         </is>
       </c>
+      <c r="B15" s="35" t="n"/>
+      <c r="C15" s="35" t="n"/>
+      <c r="D15" s="35" t="n"/>
+      <c r="E15" s="35" t="n"/>
+      <c r="F15" s="35" t="n"/>
+      <c r="G15" s="36" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
@@ -6220,6 +6323,12 @@
           <t xml:space="preserve">   3b. Pause State (SS = 0x02)</t>
         </is>
       </c>
+      <c r="B28" s="35" t="n"/>
+      <c r="C28" s="35" t="n"/>
+      <c r="D28" s="35" t="n"/>
+      <c r="E28" s="35" t="n"/>
+      <c r="F28" s="35" t="n"/>
+      <c r="G28" s="36" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
@@ -6334,6 +6443,12 @@
           <t xml:space="preserve">   3c. Error State (SS = 0x03)</t>
         </is>
       </c>
+      <c r="B33" s="35" t="n"/>
+      <c r="C33" s="35" t="n"/>
+      <c r="D33" s="35" t="n"/>
+      <c r="E33" s="35" t="n"/>
+      <c r="F33" s="35" t="n"/>
+      <c r="G33" s="36" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
@@ -6444,6 +6559,12 @@
           <t>4. AL GET  |  opcode 0x13  |  substate 0x01  |  App → Board  |  No TLVs — board replies with opcode 0x12</t>
         </is>
       </c>
+      <c r="B38" s="35" t="n"/>
+      <c r="C38" s="35" t="n"/>
+      <c r="D38" s="35" t="n"/>
+      <c r="E38" s="35" t="n"/>
+      <c r="F38" s="35" t="n"/>
+      <c r="G38" s="36" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
@@ -6464,6 +6585,12 @@
           <t>5. AL SAVE  |  opcode 0x11  |  substate 0x01  |  App → Board  |  Saves AL settings to EEPROM</t>
         </is>
       </c>
+      <c r="B41" s="35" t="n"/>
+      <c r="C41" s="35" t="n"/>
+      <c r="D41" s="35" t="n"/>
+      <c r="E41" s="35" t="n"/>
+      <c r="F41" s="35" t="n"/>
+      <c r="G41" s="36" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
@@ -6685,6 +6812,12 @@
           <t>6. AL Response  |  opcode 0x12  |  Board → App  |  Board echoes AL settings (after GET or SAVE)</t>
         </is>
       </c>
+      <c r="B49" s="35" t="n"/>
+      <c r="C49" s="35" t="n"/>
+      <c r="D49" s="35" t="n"/>
+      <c r="E49" s="35" t="n"/>
+      <c r="F49" s="35" t="n"/>
+      <c r="G49" s="36" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr">
@@ -6705,6 +6838,12 @@
           <t>7. Auto Leveller Toggle  |  opcode 0x16  |  App → Board  |  No TLVs</t>
         </is>
       </c>
+      <c r="B52" s="35" t="n"/>
+      <c r="C52" s="35" t="n"/>
+      <c r="D52" s="35" t="n"/>
+      <c r="E52" s="35" t="n"/>
+      <c r="F52" s="35" t="n"/>
+      <c r="G52" s="36" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -6746,6 +6885,12 @@
           <t>8. AL Calibration  |  opcode 0x04  |  App → Board  |  Open-loop ADC calibration</t>
         </is>
       </c>
+      <c r="B56" s="35" t="n"/>
+      <c r="C56" s="35" t="n"/>
+      <c r="D56" s="35" t="n"/>
+      <c r="E56" s="35" t="n"/>
+      <c r="F56" s="35" t="n"/>
+      <c r="G56" s="36" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
@@ -6840,6 +6985,12 @@
           <t>9. AL Calibration Result  |  opcode 0x15  |  Board → App</t>
         </is>
       </c>
+      <c r="B61" s="35" t="n"/>
+      <c r="C61" s="35" t="n"/>
+      <c r="D61" s="35" t="n"/>
+      <c r="E61" s="35" t="n"/>
+      <c r="F61" s="35" t="n"/>
+      <c r="G61" s="36" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
@@ -6958,6 +7109,12 @@
           <t>10. Motor IDs (used in Carousel Request SS field and Diagnosis TLV 0x40)</t>
         </is>
       </c>
+      <c r="B66" s="35" t="n"/>
+      <c r="C66" s="35" t="n"/>
+      <c r="D66" s="35" t="n"/>
+      <c r="E66" s="35" t="n"/>
+      <c r="F66" s="35" t="n"/>
+      <c r="G66" s="36" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -7121,6 +7278,12 @@
           <t>1. Settings From App  |  opcode 0x01  |  substate 0x00=Save  0x01=Update  |  App → Board</t>
         </is>
       </c>
+      <c r="B2" s="35" t="n"/>
+      <c r="C2" s="35" t="n"/>
+      <c r="D2" s="35" t="n"/>
+      <c r="E2" s="35" t="n"/>
+      <c r="F2" s="35" t="n"/>
+      <c r="G2" s="36" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -7461,6 +7624,12 @@
           <t>2. Settings To App  |  opcode 0x02  |  Board → App  |  Same TLV codes (0x80–0x87)</t>
         </is>
       </c>
+      <c r="B13" s="35" t="n"/>
+      <c r="C13" s="35" t="n"/>
+      <c r="D13" s="35" t="n"/>
+      <c r="E13" s="35" t="n"/>
+      <c r="F13" s="35" t="n"/>
+      <c r="G13" s="36" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
@@ -7481,6 +7650,12 @@
           <t>3. Machine State  |  opcode 0x06  |  Board → App</t>
         </is>
       </c>
+      <c r="B16" s="35" t="n"/>
+      <c r="C16" s="35" t="n"/>
+      <c r="D16" s="35" t="n"/>
+      <c r="E16" s="35" t="n"/>
+      <c r="F16" s="35" t="n"/>
+      <c r="G16" s="36" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="20" t="inlineStr">
@@ -7488,6 +7663,12 @@
           <t xml:space="preserve">   3a. Running State (SS = 0x01)</t>
         </is>
       </c>
+      <c r="B17" s="35" t="n"/>
+      <c r="C17" s="35" t="n"/>
+      <c r="D17" s="35" t="n"/>
+      <c r="E17" s="35" t="n"/>
+      <c r="F17" s="35" t="n"/>
+      <c r="G17" s="36" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="21" t="inlineStr">
@@ -7878,6 +8059,12 @@
           <t xml:space="preserve">   3b. Pause State (SS = 0x02)</t>
         </is>
       </c>
+      <c r="B30" s="35" t="n"/>
+      <c r="C30" s="35" t="n"/>
+      <c r="D30" s="35" t="n"/>
+      <c r="E30" s="35" t="n"/>
+      <c r="F30" s="35" t="n"/>
+      <c r="G30" s="36" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="21" t="inlineStr">
@@ -7955,6 +8142,12 @@
           <t xml:space="preserve">   3c. Error State (SS = 0x03)</t>
         </is>
       </c>
+      <c r="B34" s="35" t="n"/>
+      <c r="C34" s="35" t="n"/>
+      <c r="D34" s="35" t="n"/>
+      <c r="E34" s="35" t="n"/>
+      <c r="F34" s="35" t="n"/>
+      <c r="G34" s="36" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="21" t="inlineStr">
@@ -8098,6 +8291,12 @@
           <t>4. Internal Parameters (calculated in app, not sent over BT)</t>
         </is>
       </c>
+      <c r="B40" s="35" t="n"/>
+      <c r="C40" s="35" t="n"/>
+      <c r="D40" s="35" t="n"/>
+      <c r="E40" s="35" t="n"/>
+      <c r="F40" s="35" t="n"/>
+      <c r="G40" s="36" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="12" t="inlineStr">
@@ -8308,6 +8507,12 @@
           <t>5. Motor IDs (Carousel Request SS and Diagnosis TLV 0x40)</t>
         </is>
       </c>
+      <c r="B49" s="35" t="n"/>
+      <c r="C49" s="35" t="n"/>
+      <c r="D49" s="35" t="n"/>
+      <c r="E49" s="35" t="n"/>
+      <c r="F49" s="35" t="n"/>
+      <c r="G49" s="36" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -8495,8 +8700,8 @@
   <mergeCells count="9">
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A40:G40"/>
     <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A40:G40"/>
     <mergeCell ref="A34:G34"/>
     <mergeCell ref="A30:G30"/>
     <mergeCell ref="A16:G16"/>
@@ -8538,6 +8743,12 @@
           <t>1. Settings From App  |  opcode 0x01  |  substate 0x01=Update  |  App → Board</t>
         </is>
       </c>
+      <c r="B2" s="35" t="n"/>
+      <c r="C2" s="35" t="n"/>
+      <c r="D2" s="35" t="n"/>
+      <c r="E2" s="35" t="n"/>
+      <c r="F2" s="35" t="n"/>
+      <c r="G2" s="36" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="24" t="inlineStr">
@@ -9057,12 +9268,19 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="23" t="inlineStr">
         <is>
           <t>2. Settings To App  |  opcode 0x02  |  Board → App  |  Same TLV codes (0x50–0x62)</t>
         </is>
       </c>
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="35" t="n"/>
+      <c r="D18" s="35" t="n"/>
+      <c r="E18" s="35" t="n"/>
+      <c r="F18" s="35" t="n"/>
+      <c r="G18" s="36" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -9077,12 +9295,19 @@
       <c r="F19" s="8" t="inlineStr"/>
       <c r="G19" s="8" t="inlineStr"/>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="23" t="inlineStr">
         <is>
           <t>3. Machine State  |  opcode 0x06  |  Board → App</t>
         </is>
       </c>
+      <c r="B21" s="35" t="n"/>
+      <c r="C21" s="35" t="n"/>
+      <c r="D21" s="35" t="n"/>
+      <c r="E21" s="35" t="n"/>
+      <c r="F21" s="35" t="n"/>
+      <c r="G21" s="36" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="26" t="inlineStr">
@@ -9090,6 +9315,12 @@
           <t xml:space="preserve">   3a. Running / Homing State (SS = 0x01 / 0x04)</t>
         </is>
       </c>
+      <c r="B22" s="35" t="n"/>
+      <c r="C22" s="35" t="n"/>
+      <c r="D22" s="35" t="n"/>
+      <c r="E22" s="35" t="n"/>
+      <c r="F22" s="35" t="n"/>
+      <c r="G22" s="36" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
@@ -9552,12 +9783,19 @@
       </c>
       <c r="G35" s="7" t="inlineStr"/>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">   3b. Pause State (SS = 0x02)</t>
         </is>
       </c>
+      <c r="B37" s="35" t="n"/>
+      <c r="C37" s="35" t="n"/>
+      <c r="D37" s="35" t="n"/>
+      <c r="E37" s="35" t="n"/>
+      <c r="F37" s="35" t="n"/>
+      <c r="G37" s="36" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
@@ -9619,7 +9857,7 @@
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>1=UserPaused,2=SliverCut,3=LiftFault,4=BobbinFull</t>
+          <t>1=UserPaused,2=FrontSensorCut,4=Lapping,5=BackSensorCut</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -9627,7 +9865,11 @@
           <t>pauseReason</t>
         </is>
       </c>
-      <c r="G39" s="8" t="inlineStr"/>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Code 3 is unused. Confirmed against firmware #defines (BT_PAUSE_USER_PRESSED/FRONT_SENSOR_CUT/LAPPING/BACK_SENSOR_CUT) 2026-08-07 -- previous doc value (3=LiftFault,4=BobbinFull) was stale.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -9668,6 +9910,12 @@
           <t xml:space="preserve">   3c. Error State (SS = 0x03)</t>
         </is>
       </c>
+      <c r="B42" s="35" t="n"/>
+      <c r="C42" s="35" t="n"/>
+      <c r="D42" s="35" t="n"/>
+      <c r="E42" s="35" t="n"/>
+      <c r="F42" s="35" t="n"/>
+      <c r="G42" s="36" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
@@ -9844,6 +10092,12 @@
           <t>4. Reset Cut Counts  |  opcode 0x11  |  substate 0x00  |  App → Board  |  No TLVs</t>
         </is>
       </c>
+      <c r="B49" s="35" t="n"/>
+      <c r="C49" s="35" t="n"/>
+      <c r="D49" s="35" t="n"/>
+      <c r="E49" s="35" t="n"/>
+      <c r="F49" s="35" t="n"/>
+      <c r="G49" s="36" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="15" t="inlineStr">
@@ -9876,6 +10130,12 @@
           <t>5. Gearbox  |  opcode 0x08 (App→Board)  |  opcode 0x09 (Board→App)</t>
         </is>
       </c>
+      <c r="B52" s="35" t="n"/>
+      <c r="C52" s="35" t="n"/>
+      <c r="D52" s="35" t="n"/>
+      <c r="E52" s="35" t="n"/>
+      <c r="F52" s="35" t="n"/>
+      <c r="G52" s="36" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="24" t="inlineStr">
@@ -10000,6 +10260,12 @@
           <t xml:space="preserve">   Gearbox Response  |  opcode 0x09  |  Board → App</t>
         </is>
       </c>
+      <c r="B59" s="35" t="n"/>
+      <c r="C59" s="35" t="n"/>
+      <c r="D59" s="35" t="n"/>
+      <c r="E59" s="35" t="n"/>
+      <c r="F59" s="35" t="n"/>
+      <c r="G59" s="36" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="27" t="inlineStr">
@@ -10094,6 +10360,12 @@
           <t>6. Motor IDs (Carousel Request SS and Diagnosis TLV 0x40)</t>
         </is>
       </c>
+      <c r="B64" s="35" t="n"/>
+      <c r="C64" s="35" t="n"/>
+      <c r="D64" s="35" t="n"/>
+      <c r="E64" s="35" t="n"/>
+      <c r="F64" s="35" t="n"/>
+      <c r="G64" s="36" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -10343,6 +10615,12 @@
           <t>1. Settings From App  |  opcode 0x01  |  substate 0x01  |  App → Board</t>
         </is>
       </c>
+      <c r="B2" s="35" t="n"/>
+      <c r="C2" s="35" t="n"/>
+      <c r="D2" s="35" t="n"/>
+      <c r="E2" s="35" t="n"/>
+      <c r="F2" s="35" t="n"/>
+      <c r="G2" s="36" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
@@ -10683,6 +10961,12 @@
           <t>2. Settings To App  |  opcode 0x02  |  Board → App  |  Same TLV codes (0x90–0x97)</t>
         </is>
       </c>
+      <c r="B13" s="35" t="n"/>
+      <c r="C13" s="35" t="n"/>
+      <c r="D13" s="35" t="n"/>
+      <c r="E13" s="35" t="n"/>
+      <c r="F13" s="35" t="n"/>
+      <c r="G13" s="36" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="29" t="inlineStr">
@@ -10703,6 +10987,12 @@
           <t>3. Machine State  |  opcode 0x06  |  Board → App</t>
         </is>
       </c>
+      <c r="B16" s="35" t="n"/>
+      <c r="C16" s="35" t="n"/>
+      <c r="D16" s="35" t="n"/>
+      <c r="E16" s="35" t="n"/>
+      <c r="F16" s="35" t="n"/>
+      <c r="G16" s="36" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="31" t="inlineStr">
@@ -10710,6 +11000,12 @@
           <t xml:space="preserve">   3a. Running State (SS = 0x01)</t>
         </is>
       </c>
+      <c r="B17" s="35" t="n"/>
+      <c r="C17" s="35" t="n"/>
+      <c r="D17" s="35" t="n"/>
+      <c r="E17" s="35" t="n"/>
+      <c r="F17" s="35" t="n"/>
+      <c r="G17" s="36" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="32" t="inlineStr">
@@ -11026,6 +11322,12 @@
           <t xml:space="preserve">   3b. Pause State (SS = 0x02)</t>
         </is>
       </c>
+      <c r="B28" s="35" t="n"/>
+      <c r="C28" s="35" t="n"/>
+      <c r="D28" s="35" t="n"/>
+      <c r="E28" s="35" t="n"/>
+      <c r="F28" s="35" t="n"/>
+      <c r="G28" s="36" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="32" t="inlineStr">
@@ -11103,6 +11405,12 @@
           <t xml:space="preserve">   3c. Error State (SS = 0x03)</t>
         </is>
       </c>
+      <c r="B32" s="35" t="n"/>
+      <c r="C32" s="35" t="n"/>
+      <c r="D32" s="35" t="n"/>
+      <c r="E32" s="35" t="n"/>
+      <c r="F32" s="35" t="n"/>
+      <c r="G32" s="36" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="32" t="inlineStr">
@@ -11213,6 +11521,12 @@
           <t>4. Reset Grams Per Spindle  |  opcode 0x0A  |  substate 0x00  |  App → Board  |  No TLVs</t>
         </is>
       </c>
+      <c r="B37" s="35" t="n"/>
+      <c r="C37" s="35" t="n"/>
+      <c r="D37" s="35" t="n"/>
+      <c r="E37" s="35" t="n"/>
+      <c r="F37" s="35" t="n"/>
+      <c r="G37" s="36" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="30" t="inlineStr">
@@ -11237,6 +11551,12 @@
           <t>5. Output Yarn Diameter Auto-Calculation (App-side formula)</t>
         </is>
       </c>
+      <c r="B40" s="35" t="n"/>
+      <c r="C40" s="35" t="n"/>
+      <c r="D40" s="35" t="n"/>
+      <c r="E40" s="35" t="n"/>
+      <c r="F40" s="35" t="n"/>
+      <c r="G40" s="36" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="29" t="inlineStr">
@@ -11261,6 +11581,12 @@
           <t>6. Motor IDs (Carousel Request SS and Diagnosis TLV 0x40)</t>
         </is>
       </c>
+      <c r="B43" s="35" t="n"/>
+      <c r="C43" s="35" t="n"/>
+      <c r="D43" s="35" t="n"/>
+      <c r="E43" s="35" t="n"/>
+      <c r="F43" s="35" t="n"/>
+      <c r="G43" s="36" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -11377,8 +11703,8 @@
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A40:G40"/>
     <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A40:G40"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A43:G43"/>
@@ -11420,6 +11746,12 @@
           <t>Start Diagnosis  |  opcode 0x04  |  substate 0x01  |  App → Board</t>
         </is>
       </c>
+      <c r="B2" s="35" t="n"/>
+      <c r="C2" s="35" t="n"/>
+      <c r="D2" s="35" t="n"/>
+      <c r="E2" s="35" t="n"/>
+      <c r="F2" s="35" t="n"/>
+      <c r="G2" s="36" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="33" t="inlineStr">
@@ -11427,6 +11759,12 @@
           <t>Standard Motor (non-lift)</t>
         </is>
       </c>
+      <c r="B3" s="35" t="n"/>
+      <c r="C3" s="35" t="n"/>
+      <c r="D3" s="35" t="n"/>
+      <c r="E3" s="35" t="n"/>
+      <c r="F3" s="35" t="n"/>
+      <c r="G3" s="36" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="34" t="inlineStr">
@@ -11648,6 +11986,12 @@
           <t>Lift Motor (Flyer / Ring lift diagnosis)</t>
         </is>
       </c>
+      <c r="B11" s="35" t="n"/>
+      <c r="C11" s="35" t="n"/>
+      <c r="D11" s="35" t="n"/>
+      <c r="E11" s="35" t="n"/>
+      <c r="F11" s="35" t="n"/>
+      <c r="G11" s="36" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="34" t="inlineStr">
@@ -11828,6 +12172,12 @@
           <t>Diagnosis Response  |  opcode 0x05  |  substate 0x00  |  Board → App  (live, while running)</t>
         </is>
       </c>
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="35" t="n"/>
+      <c r="D18" s="35" t="n"/>
+      <c r="E18" s="35" t="n"/>
+      <c r="F18" s="35" t="n"/>
+      <c r="G18" s="36" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -12020,6 +12370,12 @@
           <t>Stop Diagnosis  |  opcode 0x04  |  substate 0x06  |  App → Board  |  No TLVs</t>
         </is>
       </c>
+      <c r="B25" s="35" t="n"/>
+      <c r="C25" s="35" t="n"/>
+      <c r="D25" s="35" t="n"/>
+      <c r="E25" s="35" t="n"/>
+      <c r="F25" s="35" t="n"/>
+      <c r="G25" s="36" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="25" t="inlineStr">
@@ -12052,6 +12408,12 @@
           <t>Reliability Notes</t>
         </is>
       </c>
+      <c r="B28" s="35" t="n"/>
+      <c r="C28" s="35" t="n"/>
+      <c r="D28" s="35" t="n"/>
+      <c r="E28" s="35" t="n"/>
+      <c r="F28" s="35" t="n"/>
+      <c r="G28" s="36" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -12150,6 +12512,12 @@
           <t>Carousel Request  |  opcode 0x07  |  Motor ID in SUBSTATE field  |  App → Board</t>
         </is>
       </c>
+      <c r="B2" s="35" t="n"/>
+      <c r="C2" s="35" t="n"/>
+      <c r="D2" s="35" t="n"/>
+      <c r="E2" s="35" t="n"/>
+      <c r="F2" s="35" t="n"/>
+      <c r="G2" s="36" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="25" t="inlineStr">
@@ -12187,6 +12555,12 @@
           <t>Carousel Response  |  opcode 0x07  |  Board → App  — Standard Motor Telemetry TLVs</t>
         </is>
       </c>
+      <c r="B6" s="35" t="n"/>
+      <c r="C6" s="35" t="n"/>
+      <c r="D6" s="35" t="n"/>
+      <c r="E6" s="35" t="n"/>
+      <c r="F6" s="35" t="n"/>
+      <c r="G6" s="36" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -12564,6 +12938,12 @@
           <t>Production Page Motor IDs per Machine (used in Carousel + logFetchJob cycle)</t>
         </is>
       </c>
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="35" t="n"/>
+      <c r="D18" s="35" t="n"/>
+      <c r="E18" s="35" t="n"/>
+      <c r="F18" s="35" t="n"/>
+      <c r="G18" s="36" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -12680,6 +13060,12 @@
           <t>Carousel Data Flow Notes</t>
         </is>
       </c>
+      <c r="B25" s="35" t="n"/>
+      <c r="C25" s="35" t="n"/>
+      <c r="D25" s="35" t="n"/>
+      <c r="E25" s="35" t="n"/>
+      <c r="F25" s="35" t="n"/>
+      <c r="G25" s="36" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -12815,6 +13201,12 @@
           <t>PID Request  |  opcode 0x0D  |  substate 0x00  |  App → Board</t>
         </is>
       </c>
+      <c r="B2" s="35" t="n"/>
+      <c r="C2" s="35" t="n"/>
+      <c r="D2" s="35" t="n"/>
+      <c r="E2" s="35" t="n"/>
+      <c r="F2" s="35" t="n"/>
+      <c r="G2" s="36" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -12880,6 +13272,12 @@
           <t>PID Response  |  opcode 0x0E  |  substate 0x00  |  Board → App</t>
         </is>
       </c>
+      <c r="B6" s="35" t="n"/>
+      <c r="C6" s="35" t="n"/>
+      <c r="D6" s="35" t="n"/>
+      <c r="E6" s="35" t="n"/>
+      <c r="F6" s="35" t="n"/>
+      <c r="G6" s="36" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -13072,6 +13470,12 @@
           <t>PID Update  |  opcode 0x0F  |  substate 0x00  |  App → Board  |  Same TLVs as response</t>
         </is>
       </c>
+      <c r="B13" s="35" t="n"/>
+      <c r="C13" s="35" t="n"/>
+      <c r="D13" s="35" t="n"/>
+      <c r="E13" s="35" t="n"/>
+      <c r="F13" s="35" t="n"/>
+      <c r="G13" s="36" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -13092,6 +13496,12 @@
           <t>PID Flow</t>
         </is>
       </c>
+      <c r="B16" s="35" t="n"/>
+      <c r="C16" s="35" t="n"/>
+      <c r="D16" s="35" t="n"/>
+      <c r="E16" s="35" t="n"/>
+      <c r="F16" s="35" t="n"/>
+      <c r="G16" s="36" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">

</xml_diff>